<commit_message>
Ready for second Full text screening
</commit_message>
<xml_diff>
--- a/04_fulltext/fullTextScreening.xlsx
+++ b/04_fulltext/fullTextScreening.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/arjen/kDrive/Obsidian/Literature Review MDIM/04_fulltext/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF3DDE09-82A1-8547-A5DB-D5DEF28A6990}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E68B51E-B3BC-9B4C-AA37-9990B104CB99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4440" yWindow="760" windowWidth="25800" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Full Text Scores" sheetId="1" r:id="rId1"/>
+    <sheet name="01_CoreScreening" sheetId="1" r:id="rId1"/>
     <sheet name="Exclusiecriteria" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Full Text Scores'!$A$1:$I$92</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_CoreScreening'!$A$1:$I$92</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -2408,7 +2408,7 @@
         <v>2</v>
       </c>
       <c r="H2" s="5">
-        <f>SUM(D2:G2)</f>
+        <f t="shared" ref="H2:H33" si="0">SUM(D2:G2)</f>
         <v>8</v>
       </c>
       <c r="I2" s="6"/>
@@ -2436,7 +2436,7 @@
         <v>2</v>
       </c>
       <c r="H3" s="5">
-        <f>SUM(D3:G3)</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="I3" s="10"/>
@@ -2464,7 +2464,7 @@
         <v>2</v>
       </c>
       <c r="H4" s="5">
-        <f>SUM(D4:G4)</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="I4" s="10"/>
@@ -2494,7 +2494,7 @@
         <v>2</v>
       </c>
       <c r="H5" s="5">
-        <f>SUM(D5:G5)</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="I5" s="10"/>
@@ -2524,7 +2524,7 @@
         <v>2</v>
       </c>
       <c r="H6" s="5">
-        <f>SUM(D6:G6)</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="I6" s="10"/>
@@ -2554,7 +2554,7 @@
         <v>2</v>
       </c>
       <c r="H7" s="5">
-        <f>SUM(D7:G7)</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="I7" s="10"/>
@@ -2584,7 +2584,7 @@
         <v>2</v>
       </c>
       <c r="H8" s="5">
-        <f>SUM(D8:G8)</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="I8" s="10"/>
@@ -2614,7 +2614,7 @@
         <v>2</v>
       </c>
       <c r="H9" s="5">
-        <f>SUM(D9:G9)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="I9" s="10"/>
@@ -2644,7 +2644,7 @@
         <v>2</v>
       </c>
       <c r="H10" s="5">
-        <f>SUM(D10:G10)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="I10" s="10"/>
@@ -2674,7 +2674,7 @@
         <v>1</v>
       </c>
       <c r="H11" s="5">
-        <f>SUM(D11:G11)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="I11" s="10"/>
@@ -2704,7 +2704,7 @@
         <v>2</v>
       </c>
       <c r="H12" s="5">
-        <f>SUM(D12:G12)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="I12" s="10"/>
@@ -2734,7 +2734,7 @@
         <v>2</v>
       </c>
       <c r="H13" s="5">
-        <f>SUM(D13:G13)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="I13" s="10"/>
@@ -2764,7 +2764,7 @@
         <v>2</v>
       </c>
       <c r="H14" s="5">
-        <f>SUM(D14:G14)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="I14" s="10"/>
@@ -2794,7 +2794,7 @@
         <v>2</v>
       </c>
       <c r="H15" s="5">
-        <f>SUM(D15:G15)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="I15" s="10"/>
@@ -2824,7 +2824,7 @@
         <v>2</v>
       </c>
       <c r="H16" s="5">
-        <f>SUM(D16:G16)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="I16" s="10"/>
@@ -2854,7 +2854,7 @@
         <v>2</v>
       </c>
       <c r="H17" s="5">
-        <f>SUM(D17:G17)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="I17" s="10"/>
@@ -2882,7 +2882,7 @@
         <v>2</v>
       </c>
       <c r="H18" s="5">
-        <f>SUM(D18:G18)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="I18" s="10"/>
@@ -2910,7 +2910,7 @@
         <v>2</v>
       </c>
       <c r="H19" s="5">
-        <f>SUM(D19:G19)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="I19" s="10"/>
@@ -2940,7 +2940,7 @@
         <v>1</v>
       </c>
       <c r="H20" s="5">
-        <f>SUM(D20:G20)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="I20" s="10"/>
@@ -2968,7 +2968,7 @@
         <v>1</v>
       </c>
       <c r="H21" s="5">
-        <f>SUM(D21:G21)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="I21" s="10"/>
@@ -2998,7 +2998,7 @@
         <v>2</v>
       </c>
       <c r="H22" s="5">
-        <f>SUM(D22:G22)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="I22" s="10"/>
@@ -3028,7 +3028,7 @@
         <v>2</v>
       </c>
       <c r="H23" s="5">
-        <f>SUM(D23:G23)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="I23" s="10"/>
@@ -3058,7 +3058,7 @@
         <v>2</v>
       </c>
       <c r="H24" s="5">
-        <f>SUM(D24:G24)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="I24" s="10"/>
@@ -3088,7 +3088,7 @@
         <v>2</v>
       </c>
       <c r="H25" s="5">
-        <f>SUM(D25:G25)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="I25" s="10"/>
@@ -3118,7 +3118,7 @@
         <v>2</v>
       </c>
       <c r="H26" s="5">
-        <f>SUM(D26:G26)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="I26" s="10"/>
@@ -3148,7 +3148,7 @@
         <v>2</v>
       </c>
       <c r="H27" s="5">
-        <f>SUM(D27:G27)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="I27" s="10"/>
@@ -3176,7 +3176,7 @@
         <v>2</v>
       </c>
       <c r="H28" s="5">
-        <f>SUM(D28:G28)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="I28" s="10"/>
@@ -3206,7 +3206,7 @@
         <v>2</v>
       </c>
       <c r="H29" s="5">
-        <f>SUM(D29:G29)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="I29" s="10"/>
@@ -3236,7 +3236,7 @@
         <v>2</v>
       </c>
       <c r="H30" s="5">
-        <f>SUM(D30:G30)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="I30" s="10"/>
@@ -3266,7 +3266,7 @@
         <v>2</v>
       </c>
       <c r="H31" s="5">
-        <f>SUM(D31:G31)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="I31" s="10"/>
@@ -3296,7 +3296,7 @@
         <v>2</v>
       </c>
       <c r="H32" s="5">
-        <f>SUM(D32:G32)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="I32" s="10"/>
@@ -3324,7 +3324,7 @@
         <v>1</v>
       </c>
       <c r="H33" s="5">
-        <f>SUM(D33:G33)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="I33" s="10"/>
@@ -3352,7 +3352,7 @@
         <v>2</v>
       </c>
       <c r="H34" s="5">
-        <f>SUM(D34:G34)</f>
+        <f t="shared" ref="H34:H65" si="1">SUM(D34:G34)</f>
         <v>7</v>
       </c>
       <c r="I34" s="10"/>
@@ -3382,7 +3382,7 @@
         <v>2</v>
       </c>
       <c r="H35" s="5">
-        <f>SUM(D35:G35)</f>
+        <f t="shared" si="1"/>
         <v>7</v>
       </c>
       <c r="I35" s="10"/>
@@ -3410,7 +3410,7 @@
         <v>2</v>
       </c>
       <c r="H36" s="5">
-        <f>SUM(D36:G36)</f>
+        <f t="shared" si="1"/>
         <v>7</v>
       </c>
       <c r="I36" s="10"/>
@@ -3442,7 +3442,7 @@
         <v>2</v>
       </c>
       <c r="H37" s="5">
-        <f>SUM(D37:G37)</f>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="I37" s="10"/>
@@ -3474,7 +3474,7 @@
         <v>2</v>
       </c>
       <c r="H38" s="5">
-        <f>SUM(D38:G38)</f>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="I38" s="10"/>
@@ -3504,7 +3504,7 @@
         <v>2</v>
       </c>
       <c r="H39" s="5">
-        <f>SUM(D39:G39)</f>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="I39" s="10"/>
@@ -3536,7 +3536,7 @@
         <v>2</v>
       </c>
       <c r="H40" s="5">
-        <f>SUM(D40:G40)</f>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="I40" s="10"/>
@@ -3566,7 +3566,7 @@
         <v>1</v>
       </c>
       <c r="H41" s="5">
-        <f>SUM(D41:G41)</f>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="I41" s="10"/>
@@ -3596,7 +3596,7 @@
         <v>2</v>
       </c>
       <c r="H42" s="5">
-        <f>SUM(D42:G42)</f>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="I42" s="10"/>
@@ -3628,7 +3628,7 @@
         <v>1</v>
       </c>
       <c r="H43" s="5">
-        <f>SUM(D43:G43)</f>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="I43" s="10"/>
@@ -3658,7 +3658,7 @@
         <v>2</v>
       </c>
       <c r="H44" s="5">
-        <f>SUM(D44:G44)</f>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="I44" s="10"/>
@@ -3690,7 +3690,7 @@
         <v>2</v>
       </c>
       <c r="H45" s="5">
-        <f>SUM(D45:G45)</f>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="I45" s="10"/>
@@ -3720,7 +3720,7 @@
         <v>1</v>
       </c>
       <c r="H46" s="5">
-        <f>SUM(D46:G46)</f>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="I46" s="10"/>
@@ -3750,7 +3750,7 @@
         <v>2</v>
       </c>
       <c r="H47" s="5">
-        <f>SUM(D47:G47)</f>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="I47" s="10"/>
@@ -3782,7 +3782,7 @@
         <v>2</v>
       </c>
       <c r="H48" s="5">
-        <f>SUM(D48:G48)</f>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="I48" s="10"/>
@@ -3812,7 +3812,7 @@
         <v>2</v>
       </c>
       <c r="H49" s="5">
-        <f>SUM(D49:G49)</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="I49" s="10"/>
@@ -3842,7 +3842,7 @@
         <v>1</v>
       </c>
       <c r="H50" s="5">
-        <f>SUM(D50:G50)</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="I50" s="10"/>
@@ -3872,7 +3872,7 @@
         <v>1</v>
       </c>
       <c r="H51" s="5">
-        <f>SUM(D51:G51)</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="I51" s="10"/>
@@ -3902,7 +3902,7 @@
         <v>2</v>
       </c>
       <c r="H52" s="5">
-        <f>SUM(D52:G52)</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="I52" s="10"/>
@@ -3932,7 +3932,7 @@
         <v>1</v>
       </c>
       <c r="H53" s="5">
-        <f>SUM(D53:G53)</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="I53" s="13"/>
@@ -3964,7 +3964,7 @@
         <v>1</v>
       </c>
       <c r="H54" s="5">
-        <f>SUM(D54:G54)</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="I54" s="10"/>
@@ -3994,7 +3994,7 @@
         <v>1</v>
       </c>
       <c r="H55" s="5">
-        <f>SUM(D55:G55)</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="I55" s="10"/>
@@ -4026,7 +4026,7 @@
         <v>1</v>
       </c>
       <c r="H56" s="5">
-        <f>SUM(D56:G56)</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="I56" s="10"/>
@@ -4056,7 +4056,7 @@
         <v>2</v>
       </c>
       <c r="H57" s="5">
-        <f>SUM(D57:G57)</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="I57" s="10"/>
@@ -4086,7 +4086,7 @@
         <v>1</v>
       </c>
       <c r="H58" s="5">
-        <f>SUM(D58:G58)</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="I58" s="10"/>
@@ -4118,7 +4118,7 @@
         <v>1</v>
       </c>
       <c r="H59" s="5">
-        <f>SUM(D59:G59)</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="I59" s="10"/>
@@ -4148,7 +4148,7 @@
         <v>2</v>
       </c>
       <c r="H60" s="5">
-        <f>SUM(D60:G60)</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="I60" s="10"/>
@@ -4178,7 +4178,7 @@
         <v>1</v>
       </c>
       <c r="H61" s="5">
-        <f>SUM(D61:G61)</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="I61" s="10"/>
@@ -4208,7 +4208,7 @@
         <v>1</v>
       </c>
       <c r="H62" s="5">
-        <f>SUM(D62:G62)</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="I62" s="10"/>
@@ -4240,7 +4240,7 @@
         <v>1</v>
       </c>
       <c r="H63" s="5">
-        <f>SUM(D63:G63)</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="I63" s="10"/>
@@ -4270,7 +4270,7 @@
         <v>1</v>
       </c>
       <c r="H64" s="5">
-        <f>SUM(D64:G64)</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="I64" s="10"/>
@@ -4302,7 +4302,7 @@
         <v>1</v>
       </c>
       <c r="H65" s="5">
-        <f>SUM(D65:G65)</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="I65" s="10"/>
@@ -4334,7 +4334,7 @@
         <v>2</v>
       </c>
       <c r="H66" s="5">
-        <f>SUM(D66:G66)</f>
+        <f t="shared" ref="H66:H97" si="2">SUM(D66:G66)</f>
         <v>5</v>
       </c>
       <c r="I66" s="10"/>
@@ -4366,7 +4366,7 @@
         <v>2</v>
       </c>
       <c r="H67" s="5">
-        <f>SUM(D67:G67)</f>
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
       <c r="I67" s="10"/>
@@ -4396,7 +4396,7 @@
         <v>1</v>
       </c>
       <c r="H68" s="5">
-        <f>SUM(D68:G68)</f>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
       <c r="I68" s="10"/>
@@ -4428,7 +4428,7 @@
         <v>1</v>
       </c>
       <c r="H69" s="5">
-        <f>SUM(D69:G69)</f>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
       <c r="I69" s="10"/>
@@ -4458,7 +4458,7 @@
         <v>1</v>
       </c>
       <c r="H70" s="5">
-        <f>SUM(D70:G70)</f>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
       <c r="I70" s="10"/>
@@ -4486,7 +4486,7 @@
         <v>1</v>
       </c>
       <c r="H71" s="5">
-        <f>SUM(D71:G71)</f>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
       <c r="I71" s="10"/>
@@ -4516,7 +4516,7 @@
         <v>2</v>
       </c>
       <c r="H72" s="5">
-        <f>SUM(D72:G72)</f>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
       <c r="I72" s="10"/>
@@ -4548,7 +4548,7 @@
         <v>0</v>
       </c>
       <c r="H73" s="5">
-        <f>SUM(D73:G73)</f>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
       <c r="I73" s="10"/>
@@ -4578,7 +4578,7 @@
         <v>1</v>
       </c>
       <c r="H74" s="5">
-        <f>SUM(D74:G74)</f>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
       <c r="I74" s="10"/>
@@ -4606,7 +4606,7 @@
         <v>1</v>
       </c>
       <c r="H75" s="5">
-        <f>SUM(D75:G75)</f>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
       <c r="I75" s="10"/>
@@ -4636,7 +4636,7 @@
         <v>1</v>
       </c>
       <c r="H76" s="5">
-        <f>SUM(D76:G76)</f>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
       <c r="I76" s="10"/>
@@ -4666,7 +4666,7 @@
         <v>1</v>
       </c>
       <c r="H77" s="5">
-        <f>SUM(D77:G77)</f>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
       <c r="I77" s="10"/>
@@ -4698,7 +4698,7 @@
         <v>1</v>
       </c>
       <c r="H78" s="5">
-        <f>SUM(D78:G78)</f>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
       <c r="I78" s="10"/>
@@ -4728,7 +4728,7 @@
         <v>1</v>
       </c>
       <c r="H79" s="5">
-        <f>SUM(D79:G79)</f>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
       <c r="I79" s="10"/>
@@ -4758,7 +4758,7 @@
         <v>1</v>
       </c>
       <c r="H80" s="5">
-        <f>SUM(D80:G80)</f>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
       <c r="I80" s="10"/>
@@ -4788,7 +4788,7 @@
         <v>1</v>
       </c>
       <c r="H81" s="5">
-        <f>SUM(D81:G81)</f>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
       <c r="I81" s="10"/>
@@ -4820,7 +4820,7 @@
         <v>1</v>
       </c>
       <c r="H82" s="5">
-        <f>SUM(D82:G82)</f>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
       <c r="I82" s="10"/>
@@ -4850,7 +4850,7 @@
         <v>1</v>
       </c>
       <c r="H83" s="5">
-        <f>SUM(D83:G83)</f>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
       <c r="I83" s="10"/>
@@ -4880,7 +4880,7 @@
         <v>1</v>
       </c>
       <c r="H84" s="5">
-        <f>SUM(D84:G84)</f>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
       <c r="I84" s="10"/>
@@ -4910,7 +4910,7 @@
         <v>1</v>
       </c>
       <c r="H85" s="5">
-        <f>SUM(D85:G85)</f>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
       <c r="I85" s="10"/>
@@ -4940,7 +4940,7 @@
         <v>1</v>
       </c>
       <c r="H86" s="5">
-        <f>SUM(D86:G86)</f>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
       <c r="I86" s="10"/>
@@ -4970,7 +4970,7 @@
         <v>1</v>
       </c>
       <c r="H87" s="5">
-        <f>SUM(D87:G87)</f>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
       <c r="I87" s="10"/>
@@ -5000,7 +5000,7 @@
         <v>1</v>
       </c>
       <c r="H88" s="5">
-        <f>SUM(D88:G88)</f>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
       <c r="I88" s="10"/>
@@ -5032,7 +5032,7 @@
         <v>1</v>
       </c>
       <c r="H89" s="5">
-        <f>SUM(D89:G89)</f>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
       <c r="I89" s="10"/>
@@ -5062,7 +5062,7 @@
         <v>1</v>
       </c>
       <c r="H90" s="5">
-        <f>SUM(D90:G90)</f>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
       <c r="I90" s="10"/>
@@ -5092,7 +5092,7 @@
         <v>1</v>
       </c>
       <c r="H91" s="5">
-        <f>SUM(D91:G91)</f>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
       <c r="I91" s="10"/>
@@ -5122,7 +5122,7 @@
         <v>1</v>
       </c>
       <c r="H92" s="5">
-        <f>SUM(D92:G92)</f>
+        <f t="shared" si="2"/>
         <v>2</v>
       </c>
       <c r="I92" s="10"/>
@@ -5175,25 +5175,25 @@
       <formula>$H2&gt;6</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J71">
-    <cfRule type="expression" dxfId="5" priority="13" stopIfTrue="1">
+  <conditionalFormatting sqref="J70">
+    <cfRule type="expression" dxfId="5" priority="1" stopIfTrue="1">
       <formula>AND($H70&lt;4,$H70&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="14" stopIfTrue="1">
+    <cfRule type="expression" dxfId="4" priority="2" stopIfTrue="1">
       <formula>AND($H70&gt;3,$H70&lt;7)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="15">
+    <cfRule type="expression" dxfId="3" priority="3">
       <formula>$H70&gt;6</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J70">
-    <cfRule type="expression" dxfId="2" priority="1" stopIfTrue="1">
+  <conditionalFormatting sqref="J71">
+    <cfRule type="expression" dxfId="2" priority="13" stopIfTrue="1">
       <formula>AND($H70&lt;4,$H70&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="2" stopIfTrue="1">
+    <cfRule type="expression" dxfId="1" priority="14" stopIfTrue="1">
       <formula>AND($H70&gt;3,$H70&lt;7)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="3">
+    <cfRule type="expression" dxfId="0" priority="15">
       <formula>$H70&gt;6</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>